<commit_message>
AI suggestions to include where suggestions are to go
</commit_message>
<xml_diff>
--- a/reports/compliance_report.xlsx
+++ b/reports/compliance_report.xlsx
@@ -428,7 +428,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="59" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -437,8 +437,8 @@
     <col width="29" customWidth="1" min="8" max="8"/>
     <col width="27" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="97" customWidth="1" min="11" max="11"/>
-    <col width="2113" customWidth="1" min="12" max="12"/>
+    <col width="173" customWidth="1" min="11" max="11"/>
+    <col width="2273" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,138 +511,129 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>185</v>
+        <v>9188</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>35.51</v>
+        <v>40.48</v>
       </c>
       <c r="G2" t="n">
-        <v>46.25</v>
+        <v>17.39</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>JTC</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Lorem ipsum</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Missing branding keywords: JTC. | Sentences are excessively long and may reduce readability.</t>
+          <t>Forbidden placeholder terms detected: Lorem ipsum. | Bullet formatting issues detected. Review bullet spacing and indentation. | High number of grammar issues detected.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Based on the issues detected in your document, here are concise suggestions to improve spacing, readability, grammar, and formatting, along with a revised version of the text.
-### Key Improvement Suggestions
-1. **Integrate Missing Keyword (JTC):** 
-   * Add context to the document by specifying that these are **JTC** application forms or part of the JTC Startup Portal.
-2. **Improve Readability &amp; Sentence Length:**
-   * Break up long, conversational sentences into shorter, professional bullet points. 
-   * Replace informal language (e.g., "vet the questions," "asks from the user," "screen grabs") with professional terms (e.g., "review," "requirements," "screenshots").
-3. **Fix Formatting &amp; Indentation:**
-   * Indent the descriptive text under items 5, 6, and 7. Currently, they look like part of the main list, which hurts visual hierarchy.
-   * Use bolding for list headers to make the document easier to scan.
-4. **Punctuation:**
-   * Add missing periods to the end of all descriptive sentences.
----
-### Revised Text (Recommended)
-&gt; **JTC Startup Portal: Form Review**
-&gt;  
-&gt; Please use the following list to review the form questions. Separate pages demonstrating the overall visual layout and design will be provided.
-&gt;  
-&gt; 1. **Startup Entity Form**
-&gt;  
-&gt; 2. **Incubator Entity Form**
-&gt;  
-&gt; 3. **Commercial Entity Form**
-&gt;  
-&gt; 4. **Step 0: Preparing Your Application**
-&gt;  
-&gt; 5. **Step 1: Application Form Header**
-&gt;    * This menu scrolls with the user to display progress and highlight incomplete mandatory fields. 
-&gt;    * The application is split into three steps to match standard JTC application flows. 
-&gt;  
-&gt; 6. **Step 1: Application Form Footer**
-&gt;    * This persistent footer allows users to save drafts at any point without scrolling. 
-&gt;    * As shown in the attached screenshots, this section remains anchored to the bottom of the screen during scrolling.
-&gt;  
-&gt; 7. **Step 2: Upload Your Documents**
-&gt;    * This step retains the original guiding text to help users navigate the extensive list of document requirements.
-&gt;  
-&gt; 8. **Step 3: Review**</t>
+          <t>Based on the review of your document, here are concise improvement suggestions organized by category to resolve formatting issues, grammatical errors, and OCR/scraping noise.
+### 1. Cleanup of OCR Noise &amp; Artifacts
+The text contains several visual artifacts, typos, and stray characters from automated scanning or scraping.
+* **Remove stray characters:** Delete random suffixes such as `e` (after *Venture Builder*), `ri)` (after *Partner)*), `Vv` (after *Singapore* and *Consumer Tech*), `Wa`, `|&lt;]`, `fi)`, and `Ke`.
+* **Fix typos:** 
+  * Change `loT` to **`IoT`** (Internet of Things).
+  * Change `feed` to **`field`** (in "*corresponding practice area / field*").
+### 2. Bullet Formatting &amp; Indentation
+* **Fix conditional logic symbols:** Replace the awkward symbols (`L&gt;`, `Ly`) used for nested questions with clean sub-bullets (e.g., `↳` or a standard indent) followed by a single space (e.g., `↳ Please specify the name of the program.`).
+* **Standardize checkboxes:** Replace raw characters like `|&lt;]` with standard checkbox symbols (e.g., `[ ] Blockchain`, `[ ] IoT`).
+### 3. Spacing &amp; Layout
+* **Clean up top spacing:** Remove the multiple consecutive blank lines at the very beginning of the document.
+* **Standardize asterisks:** Ensure there is a single space before every mandatory asterisk (e.g., change `Email*` to `Email *` and `UEN*` to `UEN *`).
+### 4. Grammar &amp; Readability
+* **Subject-verb agreement:** Change *"What problems **are** your technology solving..."* to *"What problems **is** your technology solving..."* ("technology" is singular).
+* **Fix run-on phrasing:** 
+  * Change *"Ina short and precise way..."* to *"In a concise and precise manner, describe..."* or *"Briefly describe what your company does."*
+  * Refine *"describe what your company is doing"* to *"describe what your company does"*.
+### 5. Helper Text &amp; Placeholders
+* **Differentiate helper text:** Ensure character limits (e.g., `"1000 characters left"`) and system errors (e.g., `"@ This field is required"`) are visually distinguished (italicized or bracketed) so they are not confused with form labels.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Quiz10Answers.pdf</t>
+          <t>CMD Approval - Startup (22 May) Jerron's Comments.pptx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>1251</v>
+        <v>9188</v>
       </c>
       <c r="E3" t="n">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>44.87</v>
+        <v>40.48</v>
       </c>
       <c r="G3" t="n">
-        <v>18.91</v>
+        <v>17.39</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>JTC</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lorem ipsum</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Missing branding keywords: JTC. | High number of grammar issues detected.</t>
+          <t>Forbidden placeholder terms detected: Lorem ipsum. | Bullet formatting issues detected. Review bullet spacing and indentation. | High number of grammar issues detected.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Based on the review of your document text and the detected issues, here are concise improvement suggestions categorized by key areas:
-### 1. Remove Boilerplate and Protect Privacy
-* **Remove PII:** Delete the personal login line (*"You are logged in as Jun Rong Jerron TENG (Log out)"*) to protect user privacy and make the document generalizable.
-* **Strip LMS UI Elements:** Remove system navigation elements that clutter the text (e.g., *"Data retention summary"*, *"Get the mobile app"*, and the repetitive *"Flag question"* and *"Mark x.00 out of x.00"* lines).
-* **Consolidate or Remove the Sidebar List:** The list of Questions 1 to 15 at the top takes up excessive vertical space. Delete it entirely or format it into a single-line navigation index.
-### 2. Spacing, Indentation, and Bullet Formatting
-* **Format Multiple-Choice Options:** Instead of a flat vertical list, use indented alphabetical bullets (A, B, C, D) for the answers. 
-* **Standardize Selection Markers:** Replace the raw system symbol (``) with clean, readable markers like `[Correct]` or a standard checkmark emoji (e.g., `✓ ReLU`).
-* **Group Question Blocks:** Use consistent double-line spacing between distinct questions, and single-line spacing between a question and its options to visually chunk the information.
-### 3. Readability and Grammar
-* **Clean up Metadata:** Format the test metadata (Date, Time taken, Grade) into a compact, clean table or a structured top header rather than loose lines of text.
-* **Fix Incomplete Sentences:** Complete the truncated sentence at the end: *"In a CNN, what is a "kernel" or "filter"? Choose the most appropriate **[definition/option]**."*
-* **Simplify Feedback:** Instead of repeating *"Your answer is correct. The correct answer is: [Answer]"*, use a simplified, single-line format: `Correct Answer: [Answer]`. This will drastically raise the readability score from 44.87.
-### 4. Keyword Integration (JTC)
-* **Add Missing Keyword:** Integrate the required **"JTC"** keyword naturally into the header or metadata block (e.g., *"JTC Course Portal: In-Lecture Quiz 10 [CNN]"*).</t>
+          <t>Based on the document text and the detected issues (especially the high number of grammatical errors and poor readability caused by OCR artifacts), here are concise improvement suggestions to polish your document:
+### 1. Clean Up OCR Artifacts and Garbage Characters
+* **Remove visual/OCR glitches:** Clean up trailing characters, misread checkboxes, and artifacts throughout the text:
+  * Remove `e` after "Venture Builder" and `ri)` after "Partner".
+  * Remove `Vv` after "Singapore", "Consumer Tech", and "Consumer/e-Commerce".
+  * Remove random fragments like `Wa`, `|&lt;]`, and `Ke`.
+  * Remove the trailing `fi)` after "what your company is doing. *".
+* **Trim empty lines:** Remove the excessive empty lines at the very beginning of the document.
+### 2. Standardize Formatting for Mandatory Asterisks (`*`)
+* Ensure a consistent single space before all mandatory asterisks to fix spacing issues:
+  * Change `Email*` to `Email *`
+  * Change `UEN*` to `UEN *`
+### 3. Fix Bullet Formatting and Conditional Indentations
+* **Standardize bullet markers:** Replace non-standard characters like `L&gt;` and `Ly` (used for conditional follow-up questions) with standard, clean sub-bullet points (e.g., `↳` or `◦`).
+* **Enforce bullet spacing:** Ensure there is exactly one space after every bullet or conditional arrow marker to resolve the identified bullet formatting errors (e.g., `↳ Please specify...` instead of `L&gt;Please specify...`).
+### 4. Grammar and Readability Adjustments
+* **Correct spacing typos:** 
+  * Fix `"Ina short and precise way"` to `"In a short and precise way"`.
+  * Correct `"What problems are your technology solving..."` to `"What problems **is** your technology solving..."` (or `"What problems are your technologies solving..."`).
+* **Improve flow and clarity:**
+  * For the technology tags (Blockchain, IoT, Robotics, etc.), present them as a clean, aligned checklist instead of broken lines with raw symbols.
+### 5. Final Polish of the Layout
+* Ensure clear visual hierarchy (bold headings for *Application Information*, *Eligibility Criteria*, *Company Information*, and *Business Plan*).
+* Ensure form help-text (like "1000 characters left") is italicized or styled in a smaller font to distinguish it clearly from the form field labels.</t>
         </is>
       </c>
     </row>

</xml_diff>